<commit_message>
Fix total row circular reference and format dates/columns in Excel exports
</commit_message>
<xml_diff>
--- a/Templates/Portfolio_Cedole_Template.xlsx
+++ b/Templates/Portfolio_Cedole_Template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\PerixMonitor\.0 Dati Iniziali\MP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\PerixMonitor\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D349854-76C2-4BA4-BCA6-BA0DA590DC8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0D5FE0F-0E65-477B-AE59-89E3586337B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="610" windowWidth="38620" windowHeight="21100" xr2:uid="{9D257F40-C2B9-4C7A-9E02-266CD7C5EABC}"/>
+    <workbookView xWindow="24530" yWindow="4570" windowWidth="13250" windowHeight="15430" xr2:uid="{9D257F40-C2B9-4C7A-9E02-266CD7C5EABC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -216,7 +216,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="34">
+  <dxfs count="24">
     <dxf>
       <font>
         <b/>
@@ -263,85 +263,6 @@
       <fill>
         <patternFill>
           <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFEB8953"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.89996032593768116"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
         </patternFill>
       </fill>
     </dxf>
@@ -633,17 +554,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F9038E3B-4927-4926-9484-9FEFB878B40C}" name="Table1" displayName="Table1" ref="A1:E3" totalsRowShown="0" headerRowDxfId="33" tableBorderDxfId="32">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F9038E3B-4927-4926-9484-9FEFB878B40C}" name="Table1" displayName="Table1" ref="A1:E3" totalsRowShown="0" headerRowDxfId="23" tableBorderDxfId="22">
   <autoFilter ref="A1:E3" xr:uid="{F9038E3B-4927-4926-9484-9FEFB878B40C}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E3">
     <sortCondition ref="C1:C3"/>
   </sortState>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{451A9A9B-4E9A-4A9A-A596-01758AFD54CA}" name="ISIN" dataDxfId="31"/>
-    <tableColumn id="2" xr3:uid="{4D96532D-3076-4CD2-869E-A9498CD08BAA}" name="Valore Cedola (EUR)" dataDxfId="30"/>
-    <tableColumn id="3" xr3:uid="{9E9B130A-21EB-4517-8A61-E846B7F9CB57}" name="Data Flusso" dataDxfId="29"/>
-    <tableColumn id="4" xr3:uid="{F33D46DE-BFF7-432D-9894-32D0D79A5D98}" name="Descrizione Titolo" dataDxfId="28"/>
-    <tableColumn id="5" xr3:uid="{8CEB4940-C211-46E9-92E5-B9260F06052D}" name="Fees" dataDxfId="27"/>
+    <tableColumn id="1" xr3:uid="{451A9A9B-4E9A-4A9A-A596-01758AFD54CA}" name="ISIN" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{4D96532D-3076-4CD2-869E-A9498CD08BAA}" name="Valore Cedola (EUR)" dataDxfId="20"/>
+    <tableColumn id="3" xr3:uid="{9E9B130A-21EB-4517-8A61-E846B7F9CB57}" name="Data Flusso" dataDxfId="19"/>
+    <tableColumn id="4" xr3:uid="{F33D46DE-BFF7-432D-9894-32D0D79A5D98}" name="Descrizione Titolo" dataDxfId="18"/>
+    <tableColumn id="5" xr3:uid="{8CEB4940-C211-46E9-92E5-B9260F06052D}" name="Fees" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1029,42 +950,42 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="D2:D3">
-    <cfRule type="containsText" dxfId="26" priority="52" stopIfTrue="1" operator="containsText" text="BTP">
+    <cfRule type="containsText" dxfId="16" priority="52" stopIfTrue="1" operator="containsText" text="BTP">
       <formula>NOT(ISERROR(SEARCH("BTP",D2)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="25" priority="53" stopIfTrue="1">
+    <cfRule type="expression" dxfId="15" priority="53" stopIfTrue="1">
       <formula>IF(AND(ISNUMBER(SEARCH("H2O", D2)), ISNUMBER(SEARCH("SP", D2))), 1,0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D3">
-    <cfRule type="containsText" dxfId="24" priority="42" operator="containsText" text="NEW">
+    <cfRule type="containsText" dxfId="14" priority="42" operator="containsText" text="NEW">
       <formula>NOT(ISERROR(SEARCH("NEW",D3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="23" priority="43" operator="containsText" text="Multi-Asset">
+    <cfRule type="containsText" dxfId="13" priority="43" operator="containsText" text="Multi-Asset">
       <formula>NOT(ISERROR(SEARCH("Multi-Asset",D3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="22" priority="44" operator="containsText" text="Altro">
+    <cfRule type="containsText" dxfId="12" priority="44" operator="containsText" text="Altro">
       <formula>NOT(ISERROR(SEARCH("Altro",D3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="21" priority="45" operator="containsText" text="Obbligazionario">
+    <cfRule type="containsText" dxfId="11" priority="45" operator="containsText" text="Obbligazionario">
       <formula>NOT(ISERROR(SEARCH("Obbligazionario",D3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="20" priority="46" operator="containsText" text="Obblig.">
+    <cfRule type="containsText" dxfId="10" priority="46" operator="containsText" text="Obblig.">
       <formula>NOT(ISERROR(SEARCH("Obblig.",D3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="19" priority="47" operator="containsText" text="ETF">
+    <cfRule type="containsText" dxfId="9" priority="47" operator="containsText" text="ETF">
       <formula>NOT(ISERROR(SEARCH("ETF",D3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="18" priority="48" operator="containsText" text="Azionario">
+    <cfRule type="containsText" dxfId="8" priority="48" operator="containsText" text="Azionario">
       <formula>NOT(ISERROR(SEARCH("Azionario",D3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="17" priority="49" operator="containsText" text="Liquidità">
+    <cfRule type="containsText" dxfId="7" priority="49" operator="containsText" text="Liquidità">
       <formula>NOT(ISERROR(SEARCH("Liquidità",D3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="16" priority="50" operator="containsText" text="Bilanciato">
+    <cfRule type="containsText" dxfId="6" priority="50" operator="containsText" text="Bilanciato">
       <formula>NOT(ISERROR(SEARCH("Bilanciato",D3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="15" priority="51" operator="containsText" text="Certif">
+    <cfRule type="containsText" dxfId="5" priority="51" operator="containsText" text="Certif">
       <formula>NOT(ISERROR(SEARCH("Certif",D3)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>